<commit_message>
project code and resource files
</commit_message>
<xml_diff>
--- a/project/utility/src/test/java/resources/interestRates.xlsx
+++ b/project/utility/src/test/java/resources/interestRates.xlsx
@@ -3,12 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\automation\selenium automation\seleniumAutomation\project\src\test\java\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\automation\dataDrivenTestingProject\project\utility\src\test\java\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFE1DF6F-9BB8-4FD8-BC64-AE75C0B19710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1C96C3-B319-4ACC-9B80-9E7EB782EFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
   <si>
     <t>Principle</t>
   </si>
@@ -54,9 +54,6 @@
     <t>timePeriod</t>
   </si>
   <si>
-    <t>Years</t>
-  </si>
-  <si>
     <t>Yearly</t>
   </si>
   <si>
@@ -64,6 +61,9 @@
   </si>
   <si>
     <t>Half Yearly</t>
+  </si>
+  <si>
+    <t>pass</t>
   </si>
 </sst>
 </file>
@@ -95,7 +95,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -118,6 +118,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="17"/>
       </patternFill>
     </fill>
   </fills>
@@ -148,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -165,6 +175,11 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,13 +463,13 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="13.5546875"/>
+    <col min="2" max="2" customWidth="true" width="12.0"/>
+    <col min="3" max="3" customWidth="true" width="17.44140625"/>
+    <col min="4" max="4" customWidth="true" width="14.0"/>
+    <col min="5" max="5" customWidth="true" width="16.88671875"/>
+    <col min="6" max="6" customWidth="true" width="12.0"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.33203125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
@@ -488,7 +503,7 @@
         <v>4.5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2">
         <v>10</v>
@@ -499,7 +514,9 @@
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="5"/>
+      <c r="G2" t="s" s="6">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
@@ -509,7 +526,7 @@
         <v>9.5</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D3" s="2">
         <v>9</v>
@@ -520,7 +537,9 @@
       <c r="F3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" t="s" s="7">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
@@ -541,7 +560,9 @@
       <c r="F4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" t="s" s="8">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
@@ -551,7 +572,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2">
         <v>20</v>
@@ -562,7 +583,9 @@
       <c r="F5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" t="s" s="9">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
@@ -572,7 +595,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="2">
         <v>5</v>
@@ -583,7 +606,9 @@
       <c r="F6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" t="s" s="10">
+        <v>12</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
project code and data sheet
</commit_message>
<xml_diff>
--- a/project/utility/src/test/java/resources/interestRates.xlsx
+++ b/project/utility/src/test/java/resources/interestRates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\automation\dataDrivenTestingProject\project\utility\src\test\java\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E1C96C3-B319-4ACC-9B80-9E7EB782EFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2F0A59-112C-4F6D-996A-76E2EFADE70F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="14">
   <si>
     <t>Principle</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>pass</t>
+  </si>
+  <si>
+    <t>fail</t>
   </si>
 </sst>
 </file>
@@ -95,7 +98,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -121,13 +124,23 @@
       </patternFill>
     </fill>
     <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="17"/>
+      </patternFill>
+    </fill>
+    <fill>
       <patternFill patternType="none">
         <fgColor indexed="17"/>
       </patternFill>
     </fill>
     <fill>
+      <patternFill patternType="none">
+        <fgColor indexed="10"/>
+      </patternFill>
+    </fill>
+    <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="17"/>
+        <fgColor indexed="10"/>
       </patternFill>
     </fill>
   </fills>
@@ -158,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -175,11 +188,12 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -514,7 +528,7 @@
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" t="s" s="6">
+      <c r="G2" t="s" s="7">
         <v>12</v>
       </c>
     </row>
@@ -537,7 +551,7 @@
       <c r="F3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" t="s" s="7">
+      <c r="G3" t="s" s="8">
         <v>12</v>
       </c>
     </row>
@@ -560,7 +574,7 @@
       <c r="F4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G4" t="s" s="8">
+      <c r="G4" t="s" s="9">
         <v>12</v>
       </c>
     </row>
@@ -583,7 +597,7 @@
       <c r="F5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G5" t="s" s="9">
+      <c r="G5" t="s" s="10">
         <v>12</v>
       </c>
     </row>
@@ -601,13 +615,13 @@
         <v>5</v>
       </c>
       <c r="E6" s="5">
-        <v>65717</v>
+        <v>657177777</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G6" t="s" s="10">
-        <v>12</v>
+      <c r="G6" t="s" s="11">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>